<commit_message>
refactor: change alarmliste format for printing
</commit_message>
<xml_diff>
--- a/generated/BEISPIEL_ausgabe/Luftbilanz.xlsx
+++ b/generated/BEISPIEL_ausgabe/Luftbilanz.xlsx
@@ -844,6 +844,7 @@
   <cols>
     <col width="20.6640625" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="4"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="5.5" customWidth="1" min="13" max="13"/>
     <col width="63.1640625" customWidth="1" min="14" max="14"/>
     <col width="4.83203125" customWidth="1" min="15" max="15"/>
@@ -864,7 +865,7 @@
       <c r="D2" s="38" t="n"/>
       <c r="E2" s="38" t="n"/>
     </row>
-    <row r="3" ht="17" customHeight="1">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Sanierungsobjekt:
@@ -873,11 +874,11 @@
       </c>
       <c r="C3" s="40" t="inlineStr">
         <is>
-          <t>Asbestsanierung: Asbestsanierung Küche 3 Zi.Whg. 2.OG, Worbstrasse 153, 3073 Gümligen</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Asbestsanierung: MFH Asbestsanierung Küche 3 Zi.Whg. 2.OG mit langem Beschreibungstext, Worbstrasse 153, 3073 Gümligen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">Bezeichnung Zone:
@@ -886,7 +887,7 @@
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
-          <t>Wandfliesen 25 m2</t>
+          <t>Wandfliesen 25 m2 sehr lange Beschreibung der Zone</t>
         </is>
       </c>
     </row>

</xml_diff>